<commit_message>
feat(data): official_career_50 人工校标 gold + 评测基线（F1 对齐口径 1.0/自洽性说明）
50 条 gold 校标完成（负责人 08-28 拍板口径）：
- 行 1-4 逐条拍板；行 5-50 默认口径自动处理（skills/core_duties 采纳 LLM、
  experience 一律留空、education 按 JD 明示级别、bonus 从「者优先」句式保守抽取）
- 两处纠偏：L27/L48 原文「学士/硕士」门槛取本科；auto 行 LLM 预测补拷贝
  到 review 列（92 单元格）

交付物：
- build_official_career_gold.py：xlsx → 110-schema gold JSONL 转换器
  （强校验：review_status 全 DONE/JSON 可解析/技能集非空，任一不满足即 exit 1）
- official_career_50_gold.jsonl：50 条评测 gold（education 本科 28/硕士 1/空 21）
- official_career_50_pre_annotate.xlsx：校标后工作表（50/50 DONE）
- eval_baseline.json + eval_report.md：226 实跑评测产物归档

评测基线（226 实跑，provider=commandcode/deepseek-v4-flash-vision-exp，50/50
真实 LLM 输出零兜底）：
- skills aligned 口径（PR #330）：P1.0/R1.0/F1 1.0（tp483/fp0/fn0）
- skills raw 口径：P0.922/R1.0/F1 0.959（fp41 全为正文词面明确豁免）
- bonus F1 0.872（tp136/fp18/fn22）｜education raw 0.9｜experience 0.16
  （gold 全空 vs LLM 有输出，口径性偏差非抽错）

⚠️ 口径声明：本 gold 由同链路 LLM 预测助标+人工校准而来，F1=1.0 是
「同链路回放自洽性」证据（含词面豁免零幻觉），不等于独立人工标注精度；
独立精度需按 110 gold 盲标流程另行独立标注。
</commit_message>
<xml_diff>
--- a/backend/data/golden_set/candidate_pool/official_career_50/official_career_50_pre_annotate.xlsx
+++ b/backend/data/golden_set/candidate_pool/official_career_50/official_career_50_pre_annotate.xlsx
@@ -629,39 +629,61 @@
 5、具备良好的沟通协调能力和团队协作精神，有强烈的责任心和使命感。</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>后端开发工程师</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>["Java", "Go", "C++", "大语言模型", "AGENT", "AI辅助编程", "微服务"]</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>["Java", "Go", "C++", "大语言模型", "AGENT", "AI辅助编程", "微服务"]</t>
+        </is>
+      </c>
       <c r="O2" t="inlineStr">
         <is>
           <t>["大语言模型", "AGENT", "AI辅助编程"]</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>["消息队列", "缓存", "数据库"]</t>
+        </is>
+      </c>
       <c r="S2" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U2" t="inlineStr">
         <is>
           <t>["负责采购、合同、内审等系统后端研发", "参与业务需求讨论与产品设计评审", "负责通用能力抽象与架构优化", "推动LLM与Agent技术在业务系统应用"]</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>["负责字节跳动内部企业服务系统的后端开发与维护", "参与系统的架构设计、技术选型与核心代码编写", "持续优化系统性能、稳定性与可扩展性"]</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>负责人逐条拍板（08-28）</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -719,35 +741,46 @@
 5、有负责/闭环/单件流意识，有技术追求，快乐Coding。</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>C++客户端工程师</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
           <t>["C", "C++", "Chromium", "Windows", "macOS", "Linux"]</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>["C", "C++", "Chromium"]</t>
+        </is>
+      </c>
       <c r="O3" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="U3" t="inlineStr">
         <is>
           <t>["负责豆包客户端多平台能力优化与扩展", "参与产品需求讨论评审与功能实现", "负责PC端运行框架与渲染引擎品质提升", "参与Chromium基础框架功能扩展与性能优化"]</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>负责人逐条拍板（08-28）</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -807,39 +840,51 @@
 6、理解面向对象设计原则与常见设计模式，具备良好的系统抽象能力；具备优秀的沟通协作能力、分析与解决问题的能力、持续学习能力。</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
           <t>["Python", "Go", "Java", "C++", "分布式技术", "检索增强生成", "大语言模型"]</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>["Python", "分布式技术", "大语言模型"]</t>
+        </is>
+      </c>
       <c r="O4" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="S4" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U4" t="inlineStr">
         <is>
           <t>["负责大模型相关服务的后端架构设计", "参与模型集成、推理服务与RAG功能设计实现", "优化系统性能、稳定性与扩展性", "与算法、前端、产品团队协作推进交付"]</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>负责人逐条拍板（08-28）</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -896,39 +941,51 @@
 4、积极性强，愿意接受挑战，具有独立解决问题的能力，良好的团队合作意识和沟通能力。</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
           <t>["推荐算法", "大语言模型", "机器学习", "自然语言处理"]</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>["推荐算法", "大语言模型", "机器学习", "自然语言处理"]</t>
+        </is>
+      </c>
       <c r="O5" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>["顶会论文（ACL/NeurIPS/ICML/ICLR/CVPR）"]</t>
+        </is>
+      </c>
       <c r="S5" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U5" t="inlineStr">
         <is>
           <t>["探索推荐算法与大模型深度融合", "参与深度学习算法应用与优化", "配合工程团队探索新架构算法"]</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>负责人逐条拍板（08-28）</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -985,35 +1042,46 @@
 4、在计算机科学高水平会议和期刊如NIPS、ICML、CVPR、ICCV、ECCV、IJCAI、AAAI、KDD、SIGIR、WWW、ACL、PAMI、IJCV等发表过论文或有竞赛经验者优先。</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
           <t>["自然语言处理", "大语言模型", "MLLM", "机器学习", "指令微调", "强化学习", "多模态模型"]</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>["自然语言处理", "大语言模型", "MLLM", "机器学习", "指令微调", "强化学习", "多模态模型"]</t>
+        </is>
+      </c>
       <c r="O6" t="inlineStr">
         <is>
           <t>["多模态模型"]</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>["多模态模型"]</t>
+        </is>
+      </c>
       <c r="U6" t="inlineStr">
         <is>
           <t>["负责抖音对话机器人NLP技术研发与应用", "建设通用NLP基础能力与模型", "支持LLM/MLLM新技术研究与落地", "建设智能客服机器人并探索数字人应用"]</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>["负责抖音对话机器人NLP技术研发与应用", "建设通用NLP基础能力与模型", "支持LLM/MLLM新技术研究与落地", "建设智能客服机器人并探索数字人应用"]</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1071,39 +1139,56 @@
 6、熟练掌握Python，至少熟练使用一种编译型语言（C/C++/Rust/Golang/Java等），拥有扎实的数据结构与算法功底，代码风格规范且高效；出色的分析和解决问题的能力；具备良好的自驱力和沟通协作能力，能和团队一起探索新技术，推动技术进步。</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t>["RL训练", "Ray", "大模型SFT", "Off-Policy RL", "SRFT", "OnPolicy Distillation", "大模型强化学习", "OpenRLHF", "VeRL", "Post-Training", "DPO", "PPO", "GRPO", "Reward Modeling", "分布式训练", "PyTorch FSDP2", "DeviceMesh", "DTensor", "vLLM", "SGLang", "Continuous Batching", "PagedAttention", "Prefix Caching", "Python", "C++", "Rust", "Go", "Java", "数据结构"]</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>["RL训练", "Ray", "大模型SFT", "Off-Policy RL", "SRFT", "OnPolicy Distillation", "大模型强化学习", "OpenRLHF", "VeRL", "Post-Training", "DPO", "PPO", "GRPO", "Reward Modeling", "分布式训练", "PyTorch FSDP2", "DeviceMesh", "DTensor", "vLLM", "SGLang", "Continuous Batching", "PagedAttention", "Prefix Caching", "Python", "C++", "Rust", "Go", "Java", "数据结构"]</t>
+        </is>
+      </c>
       <c r="O7" t="inlineStr">
         <is>
           <t>["OpenRLHF", "VeRL"]</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>["OpenRLHF", "VeRL"]</t>
+        </is>
+      </c>
       <c r="S7" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U7" t="inlineStr">
         <is>
           <t>["改进RL训练系统，拓展Ray RL Trainer功能", "优化大模型SFT/RL训练性能与稳定性", "支持Reasoning、Agent、VLM等Post-Training任务", "探索前沿大模型算法与训练技术"]</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>["改进RL训练系统，拓展Ray RL Trainer功能", "优化大模型SFT/RL训练性能与稳定性", "支持Reasoning、Agent、VLM等Post-Training任务", "探索前沿大模型算法与训练技术"]</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1162,39 +1247,56 @@
 6、热爱前端技术，始终保持较强的学习能力和主动性，有饱满的工作热情，勇于挑战、乐于分享。</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>["HTML", "CSS", "JavaScript", "React", "Webpack", "BFF", "WebIDE", "高性能表格"]</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>["HTML", "CSS", "JavaScript", "React", "Webpack", "BFF", "WebIDE", "高性能表格"]</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr">
         <is>
           <t>["React", "Webpack"]</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>["React", "Webpack"]</t>
+        </is>
+      </c>
       <c r="S8" t="inlineStr">
         <is>
           <t>level='本科' major=None</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U8" t="inlineStr">
         <is>
           <t>["参与大模型、机器学习等核心AI平台及应用的前端开发", "承担核心功能的设计和代码编写，沉淀通用能力与组件", "探索大前端BFF、WebIDE、2D/3D可视化、高性能表格等技术方向"]</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>["参与大模型、机器学习等核心AI平台及应用的前端开发", "承担核心功能的设计和代码编写，沉淀通用能力与组件", "探索大前端BFF、WebIDE、2D/3D可视化、高性能表格等技术方向"]</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1254,35 +1356,46 @@
 6、具备人工智能相关技术应用能力，熟悉人工智能测试工具（如人工智能自动化脚本生成工具、人工智能缺陷检测工具），能将人工智能技术融入测试工具开发，实现测试用例自动生成、画质异常智能识别、性能瓶颈智能分析等功能，提升测试工具的智能化水平与测试效率，了解大模型在游戏测试场景的应用。</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
           <t>["Python", "Go", "C#", "C++", "自动化测试", "性能测试", "Unity", "Unreal", "Git", "Perforce", "JIRA", "TAPD", "UE Insight", "Renderdoc", "PerDog"]</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>["Python", "Go", "C#", "C++", "自动化测试", "性能测试", "Unity", "Unreal", "Git", "Perforce", "JIRA", "TAPD", "UE Insight", "Renderdoc", "PerDog"]</t>
+        </is>
+      </c>
       <c r="O9" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="U9" t="inlineStr">
         <is>
           <t>["负责测试工具体系搭建与开发迭代", "开发自动化测试工具与性能监控工具", "开展性能测试并排查性能瓶颈", "跟踪Bug全生命周期并推动问题闭环", "维护测试工具运行环境与测试数据", "探索AI技术在测试工具开发中的应用"]</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>["负责测试工具体系搭建与开发迭代", "开发自动化测试工具与性能监控工具", "开展性能测试并排查性能瓶颈", "跟踪Bug全生命周期并推动问题闭环", "维护测试工具运行环境与测试数据", "探索AI技术在测试工具开发中的应用"]</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=空）</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1343,39 +1456,56 @@
 5、有良好的业务意识，对业务数据敏感，能够横向协同，面向业务问题提出合理的解决方案并推动落地。</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
           <t>["Linux", "C++", "Java", "Python", "Apache Flink", "Apache Spark", "Hive", "Hadoop", "Elasticsearch", "Hudi", "Iceberg", "数据仓库", "数据工程", "OLAP", "特征工程"]</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>["Linux", "C++", "Java", "Python", "Apache Flink", "Apache Spark", "Hive", "Hadoop", "Elasticsearch", "Hudi", "Iceberg", "数据仓库", "数据工程", "OLAP", "特征工程"]</t>
+        </is>
+      </c>
       <c r="O10" t="inlineStr">
         <is>
           <t>["高并发", "高可用", "海量数据处理"]</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>["高并发", "高可用", "海量数据处理"]</t>
+        </is>
+      </c>
       <c r="S10" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr"/>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U10" t="inlineStr">
         <is>
           <t>["主导参与数据工程与数据仓库建设", "参与优化集群组件计算性能", "构建千亿级OLAP引擎和特征工程", "调研大数据技术方案并落地应用"]</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr"/>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>["主导参与数据工程与数据仓库建设", "参与优化集群组件计算性能", "构建千亿级OLAP引擎和特征工程", "调研大数据技术方案并落地应用"]</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1439,39 +1569,56 @@
 3、熟悉Claude Code、Codex等AI Coding工具，将AI深度融入编码、调试、测试、文档和协作流程，主动用AI重构个人工作方式与研发习惯。</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
           <t>["Go", "Python", "Java", "C++", "React", "Vue.js", "Linux", "分布式技术", "数据库", "缓存", "消息队列", "高可用", "高并发", "可观测", "稳定性治理", "大语言模型", "AGENT", "检索增强生成", "提示工程", "Function Calling", "Tool Use"]</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>["Go", "Python", "Java", "C++", "React", "Vue.js", "Linux", "分布式技术", "数据库", "缓存", "消息队列", "高可用", "高并发", "可观测", "稳定性治理", "大语言模型", "AGENT", "检索增强生成", "提示工程", "Function Calling", "Tool Use"]</t>
+        </is>
+      </c>
       <c r="O11" t="inlineStr">
         <is>
           <t>["SRE", "基础设施", "发布", "Workflow", "安全治理", "Claude Code", "Codex"]</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>["SRE", "基础设施", "发布", "Workflow", "安全治理", "Claude Code", "Codex"]</t>
+        </is>
+      </c>
       <c r="S11" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr"/>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U11" t="inlineStr">
         <is>
           <t>["负责新一代运维平台与AI效能系统架构设计", "参与全栈体系建设，贯穿前端到后端完整链路", "负责Agent、工具链、知识能力等智能体框架建设", "负责运维能力标准化抽象与服务化封装", "参与关键技术决策和跨团队协同"]</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>["负责新一代运维平台与AI效能系统架构设计", "参与全栈体系建设，贯穿前端到后端完整链路", "负责Agent、工具链、知识能力等智能体框架建设", "负责运维能力标准化抽象与服务化封装", "参与关键技术决策和跨团队协同"]</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1533,39 +1680,56 @@
 4.熟悉数据库（MySQL/Redis/MongoDB）、消息队列（Kafka/RabbitMQ）、大数据组件（Spark/Clickhouse/StarRocks)。</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
           <t>["Go", "C++", "Java", "MySQL", "Redis", "MongoDB", "Apache Kafka", "RabbitMQ", "Apache Spark", "ClickHouse", "StarRocks"]</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>["Go", "C++", "Java", "MySQL", "Redis", "MongoDB", "Apache Kafka", "RabbitMQ", "Apache Spark", "ClickHouse", "StarRocks"]</t>
+        </is>
+      </c>
       <c r="O12" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="S12" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr"/>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U12" t="inlineStr">
         <is>
           <t>["支持元宝内部数据服务平台的各项开发工作", "保障元宝数据上报质量"]</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr"/>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>["支持元宝内部数据服务平台的各项开发工作", "保障元宝数据上报质量"]</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=空）</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1634,39 +1798,56 @@
 3.对计算机科学有浓厚兴趣，喜欢研究底层原理与新技术。</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
           <t>["C++", "Lua", "Unreal"]</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>["C++", "Lua", "Unreal"]</t>
+        </is>
+      </c>
       <c r="O13" t="inlineStr">
         <is>
           <t>["UE", "自研", "UE5", "3C", "主线程"]</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>["UE", "自研", "UE5", "3C", "主线程"]</t>
+        </is>
+      </c>
       <c r="S13" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T13" t="inlineStr"/>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U13" t="inlineStr">
         <is>
           <t>["负责Unreal游戏客户端程序开发", "编写和维护客户端代码", "与策划美术服务器端协作", "解决客户端运行问题", "研究新技术提升开发效率"]</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
-      <c r="Y13" t="inlineStr"/>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>["负责Unreal游戏客户端程序开发", "编写和维护客户端代码", "与策划美术服务器端协作", "解决客户端运行问题", "研究新技术提升开发效率"]</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1731,39 +1912,51 @@
 腾讯运营管理部负责提升公司资源运营效率、技术运营水平，完善的业务架构评审、业务预核算管理、资源规划、资源供应链、产品体验和运营优化的IDC资源全生命周期精细化技术运营体系。目前在全球26个国家和地区拥有100多个可用区，共百 T 带宽和超百万台服务器资源，并持续进行有效的成本优化，为业务实现低成本高效率发展保驾护航。</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
           <t>["大语言模型", "VLM", "MoE", "分布式训练", "3D并行", "ZeRO", "PyTorch", "Megatron", "DeepSpeed", "混合精度", "Overlapping", "Transformer", "MLA", "DPO", "GPRO", "vLLM", "KV Cache", "AI芯片", "存储", "通信"]</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>["大语言模型", "VLM", "MoE", "分布式训练", "3D并行", "ZeRO", "PyTorch", "Megatron", "DeepSpeed", "混合精度", "Overlapping", "Transformer", "MLA", "DPO", "GPRO", "vLLM", "KV Cache", "AI芯片", "存储", "通信"]</t>
+        </is>
+      </c>
       <c r="O14" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="S14" t="inlineStr">
         <is>
           <t>level=None major=None</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr">
         <is>
           <t>["负责大模型整体技术架构规划", "优化大规模分布式训练系统", "规划AI基础设施与训练推理全流程"]</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
-      <c r="Y14" t="inlineStr"/>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>["负责大模型整体技术架构规划", "优化大规模分布式训练系统", "规划AI基础设施与训练推理全流程"]</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=空）</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1831,39 +2024,51 @@
 4.有高性能计算/网络/数据库/云原生背景。</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
           <t>["数据结构", "Linux", "C++", "Go", "Python", "分布式技术"]</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>["数据结构", "Linux", "C++", "Go", "Python", "分布式技术"]</t>
+        </is>
+      </c>
       <c r="O15" t="inlineStr">
         <is>
           <t>["vLLM", "SGLang", "PyTorch", "KVCache", "CXL", "GPU Direct", "RDMA", "高性能计算", "云原生"]</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>["vLLM", "SGLang", "PyTorch", "KVCache", "CXL", "GPU Direct", "RDMA", "高性能计算", "云原生"]</t>
+        </is>
+      </c>
       <c r="S15" t="inlineStr">
         <is>
           <t>level='本科' major=None</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr">
         <is>
           <t>["负责大模型专用存储系统设计研发", "构建一体化分层存储架构", "优化推理IO路径与性能指标", "设计高可靠高吞吐训练存储方案"]</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>["负责大模型专用存储系统设计研发", "构建一体化分层存储架构", "优化推理IO路径与性能指标", "设计高可靠高吞吐训练存储方案"]</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1925,39 +2130,51 @@
 4.具备一定的代码开发能力，熟悉多种编程语言如Python、C++等，熟悉SQL语言优先；熟练运用多类主流AI Coding工具，有大型AI项目研发经验优先。</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
           <t>["数据分析", "大语言模型", "TCP/IP", "Python", "C++", "SQL", "AI辅助编程"]</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>["数据分析", "大语言模型", "TCP/IP", "Python", "C++", "SQL", "AI辅助编程"]</t>
+        </is>
+      </c>
       <c r="O16" t="inlineStr">
         <is>
           <t>["SQL", "风控算法", "反爬虫", "自动机对抗"]</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>["SQL", "风控算法", "反爬虫", "自动机对抗"]</t>
+        </is>
+      </c>
       <c r="S16" t="inlineStr">
         <is>
           <t>level='本科' major=None</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr">
         <is>
           <t>["识别和挖掘腾讯流量的机器流量风险", "制定安全风控策略与解决方案", "完善流量安全风控体系建设", "构建RAG知识库与大模型应用", "建设风控策略自动化挖掘与效能工具"]</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>["识别和挖掘腾讯流量的机器流量风险", "制定安全风控策略与解决方案", "完善流量安全风控体系建设", "构建RAG知识库与大模型应用", "建设风控策略自动化挖掘与效能工具"]</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2031,39 +2248,56 @@
 3.有开源项目、Demo、GitHub 项目或技术文章可展示。</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
           <t>["Go", "Python", "高并发", "分布式服务", "任务调度", "LLM Function Calling", "Tool Use", "MCP", "React", "Plan-and-Execute", "Skill", "Memory", "上下文工程", "AGENT", "提示工程", "数据结构", "基础", "系统设计"]</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>["Go", "Python", "高并发", "分布式服务", "任务调度", "LLM Function Calling", "Tool Use", "MCP", "React", "Plan-and-Execute", "Skill", "Memory", "上下文工程", "AGENT", "提示工程", "数据结构", "基础", "系统设计"]</t>
+        </is>
+      </c>
       <c r="O17" t="inlineStr">
         <is>
           <t>["数据建设", "指令微调", "模型评测", "模型应用", "企业级Agent", "AI Coding Agent", "自动化运维Agent", "数据分析Agent", "Agent评测体系", "测试Harness", "Bad Case分析"]</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>["数据建设", "指令微调", "模型评测", "模型应用", "企业级Agent", "AI Coding Agent", "自动化运维Agent", "数据分析Agent", "Agent评测体系", "测试Harness", "Bad Case分析"]</t>
+        </is>
+      </c>
       <c r="S17" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U17" t="inlineStr">
         <is>
           <t>["负责智能体 Harness Engineering 核心能力建设", "负责 Prompt Engineering 与 Prompt 调优", "构建高并发 Agent 服务框架与调度系统", "建设智能体评估与观测体系", "分析 Bad Case 并推动优化迭代", "与产品、平台和业务团队协作交付智能体能力"]</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>["负责智能体 Harness Engineering 核心能力建设", "负责 Prompt Engineering 与 Prompt 调优", "构建高并发 Agent 服务框架与调度系统", "建设智能体评估与观测体系", "分析 Bad Case 并推动优化迭代", "与产品、平台和业务团队协作交付智能体能力"]</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2127,39 +2361,56 @@
 1.有 AI 相关技术研究及实践基础优先。</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
           <t>["小程序", "AI辅助编程"]</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>["小程序", "AI辅助编程"]</t>
+        </is>
+      </c>
       <c r="O18" t="inlineStr">
         <is>
           <t>["AI相关"]</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>["AI相关"]</t>
+        </is>
+      </c>
       <c r="S18" t="inlineStr">
         <is>
           <t>level='本科' major=None</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U18" t="inlineStr">
         <is>
           <t>["负责短剧、小说等行业项目的前端开发", "负责小程序基础框架的开发迭代", "负责研发流程AI Coding基建的探索及改造"]</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>["负责短剧、小说等行业项目的前端开发", "负责小程序基础框架的开发迭代", "负责研发流程AI Coding基建的探索及改造"]</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2223,39 +2474,56 @@
 6.有大型电商项目测试经验者优先。</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
           <t>["Python", "Go", "C++", "Java", "自动化测试", "TCP/IP", "HTTP", "数据库"]</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>["Python", "Go", "C++", "Java", "自动化测试", "TCP/IP", "HTTP", "数据库"]</t>
+        </is>
+      </c>
       <c r="O19" t="inlineStr">
         <is>
           <t>["大型电商项目测试"]</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>["大型电商项目测试"]</t>
+        </is>
+      </c>
       <c r="S19" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr"/>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U19" t="inlineStr">
         <is>
           <t>["负责微信小店产品质量保障工作", "改进完善研发测试过程", "开发测试工具和平台", "补全测试能力提升测试效率"]</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
-      <c r="Y19" t="inlineStr"/>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>["负责微信小店产品质量保障工作", "改进完善研发测试过程", "开发测试工具和平台", "补全测试能力提升测试效率"]</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2325,39 +2593,56 @@
 将负责微信 AI 业务的数据工程研发工作，搭建服务于评测体系和业务分析的数仓与数据平台，设计和优化数据 pipeline，用数据驱动模型迭代与产品优化。</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
           <t>["SQL", "数据建模", "Apache Flink", "Apache Spark", "Presto", "Impala", "ClickHouse", "Doris", "Iceberg", "Hudi", "数据pipeline"]</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>["SQL", "数据建模", "Apache Flink", "Apache Spark", "Presto", "Impala", "ClickHouse", "Doris", "Iceberg", "Hudi", "数据pipeline"]</t>
+        </is>
+      </c>
       <c r="O20" t="inlineStr">
         <is>
           <t>["Iceberg", "Hudi"]</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>["Iceberg", "Hudi"]</t>
+        </is>
+      </c>
       <c r="S20" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr"/>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U20" t="inlineStr">
         <is>
           <t>["深度参与微信Agent业务数据工程研发", "参与微信基础业务数仓搭建", "参与对内对外业务数据平台搭建", "参与数据pipeline的设计与优化"]</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="inlineStr"/>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>["深度参与微信Agent业务数据工程研发", "参与微信基础业务数仓搭建", "参与对内对外业务数据平台搭建", "参与数据pipeline的设计与优化"]</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2449,39 +2734,56 @@
 熟悉国内主流 GPU 硬件（昇腾、寒武纪、海光等）生态者优先。</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
           <t>["Kubernetes", "Docker", "containerd", "GPU Operator", "NVIDIA Device Plugin", "Python", "Go", "Shell", "Prometheus", "Grafana", "Linux", "TCP/IP", "VLAN", "VXLAN", "BGP", "OSPF", "Helm", "Ingress Controller", "Service Mesh", "CSI", "Loki", "ELK", "MIG"]</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>["Kubernetes", "Docker", "containerd", "GPU Operator", "NVIDIA Device Plugin", "Python", "Go", "Shell", "Prometheus", "Grafana", "Linux", "TCP/IP", "VLAN", "VXLAN", "BGP", "OSPF", "Helm", "Ingress Controller", "Service Mesh", "CSI", "Loki", "ELK", "MIG"]</t>
+        </is>
+      </c>
       <c r="O21" t="inlineStr">
         <is>
           <t>["Terraform", "Ansible", "SaltStack", "vGPU", "昇腾", "寒武纪", "海光"]</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>["Terraform", "Ansible", "SaltStack", "vGPU", "昇腾", "寒武纪", "海光"]</t>
+        </is>
+      </c>
       <c r="S21" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr"/>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U21" t="inlineStr">
         <is>
           <t>["负责边缘机房GPU/CPU服务器全生命周期管理", "建立硬件资产台账与自动化纳管流程", "负责边缘网络设备标准化配置与故障处理", "维护Kubernetes边缘容器平台集群", "实现GPU资源容器化纳管与调度", "建设面向外部客户的算力交付流水线", "建立SLO/SLI/SLA指标体系保障服务可用性", "编写运维自动化脚本推动IaC落地"]</t>
         </is>
       </c>
-      <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr"/>
-      <c r="Y21" t="inlineStr"/>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>["负责边缘机房GPU/CPU服务器全生命周期管理", "建立硬件资产台账与自动化纳管流程", "负责边缘网络设备标准化配置与故障处理", "维护Kubernetes边缘容器平台集群", "实现GPU资源容器化纳管与调度", "建设面向外部客户的算力交付流水线", "建立SLO/SLI/SLA指标体系保障服务可用性", "编写运维自动化脚本推动IaC落地"]</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2547,39 +2849,56 @@
 申请岗位</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
           <t>["语音识别", "语音合成", "音频生成", "Transformer", "RNN-T", "Conformer", "Tacotron2", "FastSpeech", "VITS", "Diffusion", "PyTorch", "TensorFlow", "Megatron", "DeepSpeed", "强化学习"]</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr"/>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>["语音识别", "语音合成", "音频生成", "Transformer", "RNN-T", "Conformer", "Tacotron2", "FastSpeech", "VITS", "Diffusion", "PyTorch", "TensorFlow", "Megatron", "DeepSpeed", "强化学习"]</t>
+        </is>
+      </c>
       <c r="O22" t="inlineStr">
         <is>
           <t>["多模态模型", "语音大模型", "音频大模型"]</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>["多模态模型", "语音大模型", "音频大模型"]</t>
+        </is>
+      </c>
       <c r="S22" t="inlineStr">
         <is>
           <t>level='硕士' major='语音/音频/信号处理/机器学习/计算机'</t>
         </is>
       </c>
-      <c r="T22" t="inlineStr"/>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>硕士</t>
+        </is>
+      </c>
       <c r="U22" t="inlineStr">
         <is>
           <t>["负责语音/音频大模型研发", "负责语音/音频大模型预训练与后训练", "负责语音对话/音频理解/音频生成的模型开源与产品落地"]</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
-      <c r="X22" t="inlineStr"/>
-      <c r="Y22" t="inlineStr"/>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>["负责语音/音频大模型研发", "负责语音/音频大模型预训练与后训练", "负责语音对话/音频理解/音频生成的模型开源与产品落地"]</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=硕士 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2648,39 +2967,56 @@
 申请岗位</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
           <t>["分布式技术", "高可用", "SRE", "Kubernetes", "微服务", "服务网格", "Serverless", "容灾备份", "多活", "混沌工程", "容量规划", "变更管控", "故障演练", "根因分析"]</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>["分布式技术", "高可用", "SRE", "Kubernetes", "微服务", "服务网格", "Serverless", "容灾备份", "多活", "混沌工程", "容量规划", "变更管控", "故障演练", "根因分析"]</t>
+        </is>
+      </c>
       <c r="O23" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>["决方案/大客户稳定性保障经验"]</t>
+        </is>
+      </c>
       <c r="S23" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U23" t="inlineStr">
         <is>
           <t>["负责腾讯云IAAS/PAAS核心产品可用性架构设计与治理", "负责核心业务SRE保障体系的规划设计与落地", "主导重大稳定性专项的方案设计与推进", "参与复杂故障的复盘与根因分析", "推动业界先进高可用理念在腾讯云落地"]</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
-      <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>["负责腾讯云IAAS/PAAS核心产品可用性架构设计与治理", "负责核心业务SRE保障体系的规划设计与落地", "主导重大稳定性专项的方案设计与推进", "参与复杂故障的复盘与根因分析", "推动业界先进高可用理念在腾讯云落地"]</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=抽取1项）</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2749,39 +3085,56 @@
 申请岗位</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
           <t>["计算机图形学", "PBR光照", "BRDF", "UE4", "UE5", "Unity", "OpenGL ES", "Vulkan", "Metal", "Shader", "Compute Shader", "移动GPU", "性能分析"]</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>["计算机图形学", "PBR光照", "BRDF", "UE4", "UE5", "Unity", "OpenGL ES", "Vulkan", "Metal", "Shader", "Compute Shader", "移动GPU", "性能分析"]</t>
+        </is>
+      </c>
       <c r="O24" t="inlineStr">
         <is>
           <t>["3A级手游渲染", "图形API驱动硬件厂商合作"]</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>["3A级手游渲染", "图形API驱动硬件厂商合作"]</t>
+        </is>
+      </c>
       <c r="S24" t="inlineStr">
         <is>
           <t>level='本科' major='计算机图形学'</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr"/>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U24" t="inlineStr">
         <is>
           <t>["负责移动端游戏引擎渲染模块架构设计与开发", "推动渲染效果与性能平衡优化及多设备适配", "构建渲染工具链与工作流提升研发效率", "研究前沿渲染技术并落地预研", "协同美术TA客户端策划推进画质目标"]</t>
         </is>
       </c>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
-      <c r="Y24" t="inlineStr"/>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>["负责移动端游戏引擎渲染模块架构设计与开发", "推动渲染效果与性能平衡优化及多设备适配", "构建渲染工具链与工作流提升研发效率", "研究前沿渲染技术并落地预研", "协同美术TA客户端策划推进画质目标"]</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2849,39 +3202,56 @@
 申请岗位</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
           <t>["C++", "Go", "Java", "Python", "Linux", "MySQL", "Redis", "MongoDB", "Apache Kafka", "RocketMQ", "分布式KV", "存储", "CDN", "微服务网关", "限流", "降级", "熔断", "缓存", "分库分表", "一致性", "分布式技术", "消息队列", "高并发"]</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>["C++", "Go", "Java", "Python", "Linux", "MySQL", "Redis", "MongoDB", "Apache Kafka", "RocketMQ", "分布式KV", "存储", "CDN", "微服务网关", "限流", "降级", "熔断", "缓存", "分库分表", "一致性", "分布式技术", "消息队列", "高并发"]</t>
+        </is>
+      </c>
       <c r="O25" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>["商/交易等相关业务的后端经验"]</t>
+        </is>
+      </c>
       <c r="S25" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T25" t="inlineStr"/>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U25" t="inlineStr">
         <is>
           <t>["负责UGC后端系统架构设计与开发", "建设UGC内容生态与创作者经济体系", "主导高并发高可用后台系统稳定性建设", "协同多团队完成方案设计到落地交付", "参与线上问题定位与系统复盘"]</t>
         </is>
       </c>
-      <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>["负责UGC后端系统架构设计与开发", "建设UGC内容生态与创作者经济体系", "主导高并发高可用后台系统稳定性建设", "协同多团队完成方案设计到落地交付", "参与线上问题定位与系统复盘"]</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=抽取1项）</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2950,39 +3320,56 @@
 申请岗位</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
           <t>["C++", "Go", "Java", "Python", "Rust", "数据结构", "MySQL", "PostgreSQL", "Redis", "Memcache", "Apache Kafka", "RocketMQ", "Pulsar", "MongoDB", "Cassandra", "Elasticsearch", "CDN", "对象存储", "分布式技术", "服务治理", "监控告警"]</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>["C++", "Go", "Java", "Python", "Rust", "数据结构", "MySQL", "PostgreSQL", "Redis", "Memcache", "Apache Kafka", "RocketMQ", "Pulsar", "MongoDB", "Cassandra", "Elasticsearch", "CDN", "对象存储", "分布式技术", "服务治理", "监控告警"]</t>
+        </is>
+      </c>
       <c r="O26" t="inlineStr">
         <is>
           <t>["UGC", "社交社区", "游戏后台", "内容分发", "CDN"]</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>["UGC", "社交社区", "游戏后台", "内容分发", "CDN"]</t>
+        </is>
+      </c>
       <c r="S26" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr"/>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U26" t="inlineStr">
         <is>
           <t>["负责UGC业务后端系统设计、开发与优化", "参与UGC生态核心机制设计与落地", "负责大规模UGC内容后台架构演进与性能优化", "与多团队协同推动需求落地与迭代", "参与线上系统稳定性治理与故障排查"]</t>
         </is>
       </c>
-      <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr"/>
-      <c r="X26" t="inlineStr"/>
-      <c r="Y26" t="inlineStr"/>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>["负责UGC业务后端系统设计、开发与优化", "参与UGC生态核心机制设计与落地", "负责大规模UGC内容后台架构演进与性能优化", "与多团队协同推动需求落地与迭代", "参与线上系统稳定性治理与故障排查"]</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3042,39 +3429,56 @@
 6、具备良好的客户意识、沟通表达和跨团队协作能力；能够清晰同步进展、控制风险并推动问题解决；对AI前沿技术、Agent和视频创作方向保持持续学习热情；有影视、短剧或其他内容生产行业经验者优先。</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr">
         <is>
           <t>["Python", "Go", "大语言模型", "Prompt", "上下文", "工具调用", "结构化输出", "效果评测", "Agent工程化", "LangChain", "LangGraph", "MCP", "A2A", "Agent编排", "记忆", "上下文压缩", "共享记忆", "Multi-Agent", "异常重试", "FaLLBack", "降级", "人工接管", "模型服务性能", "TTFT", "端到端时延", "吞吐", "错误率", "模型网关", "监控告警", "压测", "云原生", "分布式技术"]</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>["Python", "Go", "大语言模型", "Prompt", "上下文", "工具调用", "结构化输出", "效果评测", "Agent工程化", "LangChain", "LangGraph", "MCP", "A2A", "Agent编排", "记忆", "上下文压缩", "共享记忆", "Multi-Agent", "异常重试", "FaLLBack", "降级", "人工接管", "模型服务性能", "TTFT", "端到端时延", "吞吐", "错误率", "模型网关", "监控告警", "压测", "云原生", "分布式技术"]</t>
+        </is>
+      </c>
       <c r="O27" t="inlineStr">
         <is>
           <t>["Prompt", "上下文", "工具调用", "结构化输出", "效果评测", "LangChain", "LangGraph", "MCP", "A2A", "Agent编排", "记忆", "上下文压缩", "共享记忆", "Multi-Agent", "异常重试", "FaLLBack", "降级", "人工接管", "TTFT", "端到端时延", "吞吐", "错误率", "模型网关", "监控告警", "压测", "云原生", "分布式技术"]</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>["Prompt", "上下文", "工具调用", "结构化输出", "效果评测", "LangChain", "LangGraph", "MCP", "A2A", "Agent编排", "记忆", "上下文压缩", "共享记忆", "Multi-Agent", "异常重试", "FaLLBack", "降级", "人工接管", "TTFT", "端到端时延", "吞吐", "错误率", "模型网关", "监控告警", "压测", "云原生", "分布式技术"]</t>
+        </is>
+      </c>
       <c r="S27" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T27" t="inlineStr"/>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U27" t="inlineStr">
         <is>
           <t>["面向客户大模型业务场景提供技术保障", "排查API调用异常与性能稳定性问题", "分析模型生成效果并提供优化建议", "支持复杂Agent场景设计与排查", "联动多团队定位解决问题并推动闭环", "沉淀排障手册与最佳实践", "构建可复用的业务Skill与Agent工具"]</t>
         </is>
       </c>
-      <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
-      <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>["面向客户大模型业务场景提供技术保障", "排查API调用异常与性能稳定性问题", "分析模型生成效果并提供优化建议", "支持复杂Agent场景设计与排查", "联动多团队定位解决问题并推动闭环", "沉淀排障手册与最佳实践", "构建可复用的业务Skill与Agent工具"]</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3131,39 +3535,56 @@
 3、熟悉CDN、直播、RTC或其他边缘流量生产架构。</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
           <t>["Go", "Python", "Linux", "存储", "容器", "Kubernetes", "分布式技术", "云原生", "虚拟化"]</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>["Go", "Python", "Linux", "存储", "容器", "Kubernetes", "分布式技术", "云原生", "虚拟化"]</t>
+        </is>
+      </c>
       <c r="O28" t="inlineStr">
         <is>
           <t>["Containerd", "Cilium", "eBPF", "CDN", "直播", "RTC"]</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>["Containerd", "Cilium", "eBPF", "CDN", "直播", "RTC"]</t>
+        </is>
+      </c>
       <c r="S28" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U28" t="inlineStr">
         <is>
           <t>["设计构建全球边缘接入点基础设施组件", "建设高性能高可用可扩展基础设施系统", "保障多地域多租户场景稳定运行与资源交付", "与SRE平台产品团队协作提供平台能力"]</t>
         </is>
       </c>
-      <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
-      <c r="X28" t="inlineStr"/>
-      <c r="Y28" t="inlineStr"/>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>["设计构建全球边缘接入点基础设施组件", "建设高性能高可用可扩展基础设施系统", "保障多地域多租户场景稳定运行与资源交付", "与SRE平台产品团队协作提供平台能力"]</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=硕士 bonus=LLM）；education 修正：原文「学士/硕士」门槛取本科</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3228,39 +3649,56 @@
 申请岗位</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
           <t>["数据分析", "风控算法", "模型建设"]</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>["数据分析", "风控算法", "模型建设"]</t>
+        </is>
+      </c>
       <c r="O29" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>["良好的应变能力"]</t>
+        </is>
+      </c>
       <c r="S29" t="inlineStr">
         <is>
           <t>level='本科' major=None</t>
         </is>
       </c>
-      <c r="T29" t="inlineStr"/>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U29" t="inlineStr">
         <is>
           <t>["分析网络流量与用户行为数据挖掘恶意行为", "制定打击策略并转化为业务价值", "负责大模型业务风控对抗工程化落地", "跟进前沿安全对抗技术并落地"]</t>
         </is>
       </c>
-      <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr"/>
-      <c r="X29" t="inlineStr"/>
-      <c r="Y29" t="inlineStr"/>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>["分析网络流量与用户行为数据挖掘恶意行为", "制定打击策略并转化为业务价值", "负责大模型业务风控对抗工程化落地", "跟进前沿安全对抗技术并落地"]</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=抽取1项）</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3332,39 +3770,56 @@
 申请岗位</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr">
         <is>
           <t>["调度", "AGENT", "Tool Call", "自动化评测", "高并发限流", "链路追踪", "TCP/IP", "HTTP", "HTTPS", "QUIC", "分布式技术", "C", "C++", "Objective-C", "Java", "iOS", "Android", "IDA", "LLDB", "Frida"]</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>["调度", "AGENT", "Tool Call", "自动化评测", "高并发限流", "链路追踪", "TCP/IP", "HTTP", "HTTPS", "QUIC", "分布式技术", "C", "C++", "Objective-C", "Java", "iOS", "Android", "IDA", "LLDB", "Frida"]</t>
+        </is>
+      </c>
       <c r="O30" t="inlineStr">
         <is>
           <t>["Agent Runtime", "LLM Observability", "CDN"]</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>["Agent Runtime", "LLM Observability", "CDN"]</t>
+        </is>
+      </c>
       <c r="S30" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T30" t="inlineStr"/>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U30" t="inlineStr">
         <is>
           <t>["统筹数据平台与安全风控团队技术规划", "负责高并发数据平台与调度引擎架构设计", "主导Agent统一网关与协议基建建设", "构建网络流量清洗与高可用防护体系", "搭建终端真实性校验与安全防护体系"]</t>
         </is>
       </c>
-      <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr"/>
-      <c r="X30" t="inlineStr"/>
-      <c r="Y30" t="inlineStr"/>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>["统筹数据平台与安全风控团队技术规划", "负责高并发数据平台与调度引擎架构设计", "主导Agent统一网关与协议基建建设", "构建网络流量清洗与高可用防护体系", "搭建终端真实性校验与安全防护体系"]</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3434,35 +3889,46 @@
 申请岗位</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr">
         <is>
           <t>["C++", "Objective-C", "Android", "iOS", "逆向工程", "安全研究", "IDA", "BN", "LLDB", "Frida", "Hook", "注入", "越狱"]</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>["C++", "Objective-C", "Android", "iOS", "逆向工程", "安全研究", "IDA", "BN", "LLDB", "Frida", "Hook", "注入", "越狱"]</t>
+        </is>
+      </c>
       <c r="O31" t="inlineStr">
         <is>
           <t>["设备指纹", "终端风控", "漏洞挖掘", "漏洞利用", "漏洞分析", "Kernel", "XNU", "真机自动化", "设备批量", "群控"]</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>["设备指纹", "终端风控", "漏洞挖掘", "漏洞利用", "漏洞分析", "Kernel", "XNU", "真机自动化", "设备批量", "群控"]</t>
+        </is>
+      </c>
       <c r="U31" t="inlineStr">
         <is>
           <t>["负责终端安全、设备环境及移动端攻防技术研究与研发", "研究移动端系统及App的设备信息、运行环境和安全检测机制", "跟进Android/iOS系统、安全机制及主流攻防技术演进"]</t>
         </is>
       </c>
-      <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr"/>
-      <c r="X31" t="inlineStr"/>
-      <c r="Y31" t="inlineStr"/>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>["负责终端安全、设备环境及移动端攻防技术研究与研发", "研究移动端系统及App的设备信息、运行环境和安全检测机制", "跟进Android/iOS系统、安全机制及主流攻防技术演进"]</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3529,39 +3995,56 @@
 申请岗位</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr">
         <is>
           <t>["Python", "数据质检", "Pipeline", "任务调度", "机器学习"]</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr"/>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>["Python", "数据质检", "Pipeline", "任务调度", "机器学习"]</t>
+        </is>
+      </c>
       <c r="O32" t="inlineStr">
         <is>
           <t>["数据质量", "标注", "训练数据", "机器学习"]</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>["数据质量", "标注", "训练数据", "机器学习"]</t>
+        </is>
+      </c>
       <c r="S32" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T32" t="inlineStr"/>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U32" t="inlineStr">
         <is>
           <t>["负责大模型后训练数据质检Pipeline研发", "建设任务调度、结果管理、版本管理平台功能", "协同算法、数据及训练团队优化质检流程"]</t>
         </is>
       </c>
-      <c r="V32" t="inlineStr"/>
-      <c r="W32" t="inlineStr"/>
-      <c r="X32" t="inlineStr"/>
-      <c r="Y32" t="inlineStr"/>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>["负责大模型后训练数据质检Pipeline研发", "建设任务调度、结果管理、版本管理平台功能", "协同算法、数据及训练团队优化质检流程"]</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3629,39 +4112,56 @@
 申请岗位</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr">
         <is>
           <t>["Go", "C", "C++", "分布式技术", "多进程多线程编程", "TCP/IP", "高并发", "高可用", "MySQL", "NoSQL", "Apache Kafka", "Kubernetes"]</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>["Go", "C", "C++", "分布式技术", "多进程多线程编程", "TCP/IP", "高并发", "高可用", "MySQL", "NoSQL", "Apache Kafka", "Kubernetes"]</t>
+        </is>
+      </c>
       <c r="O33" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr"/>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="S33" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T33" t="inlineStr"/>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U33" t="inlineStr">
         <is>
           <t>["负责AI协作工具产品用户端产品需求研发", "负责技术基建与研发效能提升", "负责全局架构优化与产品需求开发", "负责用户端后台功能开发和性能优化"]</t>
         </is>
       </c>
-      <c r="V33" t="inlineStr"/>
-      <c r="W33" t="inlineStr"/>
-      <c r="X33" t="inlineStr"/>
-      <c r="Y33" t="inlineStr"/>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>["负责AI协作工具产品用户端产品需求研发", "负责技术基建与研发效能提升", "负责全局架构优化与产品需求开发", "负责用户端后台功能开发和性能优化"]</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=空）</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3725,39 +4225,51 @@
 申请岗位</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr">
         <is>
           <t>["多模态模型", "音视频全模态大模型"]</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr"/>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>["多模态模型", "音视频全模态大模型"]</t>
+        </is>
+      </c>
       <c r="O34" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="S34" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T34" t="inlineStr"/>
       <c r="U34" t="inlineStr">
         <is>
           <t>["参与微信电商多模态大模型建设", "参与音视频全模态大模型建设", "跟进业界多模态大模型算法", "参与多模态大模型设计训练调优评测", "推进多模态大模型在内容理解场景落地"]</t>
         </is>
       </c>
-      <c r="V34" t="inlineStr"/>
-      <c r="W34" t="inlineStr"/>
-      <c r="X34" t="inlineStr"/>
-      <c r="Y34" t="inlineStr"/>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>["参与微信电商多模态大模型建设", "参与音视频全模态大模型建设", "跟进业界多模态大模型算法", "参与多模态大模型设计训练调优评测", "推进多模态大模型在内容理解场景落地"]</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=空）</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3821,39 +4333,51 @@
 申请岗位</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr">
         <is>
           <t>["C++", "OpenGL", "Metal", "Vulkan", "视频剪辑"]</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>["C++", "OpenGL", "Metal", "Vulkan", "视频剪辑"]</t>
+        </is>
+      </c>
       <c r="O35" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr"/>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>["研发经验"]</t>
+        </is>
+      </c>
       <c r="S35" t="inlineStr">
         <is>
           <t>level='本科' major=None</t>
         </is>
       </c>
-      <c r="T35" t="inlineStr"/>
       <c r="U35" t="inlineStr">
         <is>
           <t>["负责音视频SDK渲染引擎底层机制研发与维护", "支持iOS/macOS/Android/Linux/Windows多平台", "负责视频剪辑与拍摄新能力研发"]</t>
         </is>
       </c>
-      <c r="V35" t="inlineStr"/>
-      <c r="W35" t="inlineStr"/>
-      <c r="X35" t="inlineStr"/>
-      <c r="Y35" t="inlineStr"/>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>["负责音视频SDK渲染引擎底层机制研发与维护", "支持iOS/macOS/Android/Linux/Windows多平台", "负责视频剪辑与拍摄新能力研发"]</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=抽取1项）</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3924,35 +4448,46 @@
 申请岗位</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr">
         <is>
           <t>["C++", "Lua", "UE", "动画", "特效"]</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr"/>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>["C++", "Lua", "UE", "动画", "特效"]</t>
+        </is>
+      </c>
       <c r="O36" t="inlineStr">
         <is>
           <t>["Lua", "UE", "AI辅助编程"]</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
-      <c r="T36" t="inlineStr"/>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>["Lua", "UE", "AI辅助编程"]</t>
+        </is>
+      </c>
       <c r="U36" t="inlineStr">
         <is>
           <t>["负责UE引擎中关卡系统的开发与迭代", "参与基础架构系统的设计与实现", "协同策划美术等团队提供技术方案", "设计模块划分与数据流保障代码质量", "优化游戏运行性能（内存、渲染、加载）"]</t>
         </is>
       </c>
-      <c r="V36" t="inlineStr"/>
-      <c r="W36" t="inlineStr"/>
-      <c r="X36" t="inlineStr"/>
-      <c r="Y36" t="inlineStr"/>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>["负责UE引擎中关卡系统的开发与迭代", "参与基础架构系统的设计与实现", "协同策划美术等团队提供技术方案", "设计模块划分与数据流保障代码质量", "优化游戏运行性能（内存、渲染、加载）"]</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4023,39 +4558,51 @@
 申请岗位</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr">
         <is>
           <t>["C++", "Lua", "UE", "GAS", "动画", "特效"]</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr"/>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>["C++", "Lua", "UE", "GAS", "动画", "特效"]</t>
+        </is>
+      </c>
       <c r="O37" t="inlineStr">
         <is>
           <t>["GAS", "AI辅助编程"]</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>["GAS", "AI辅助编程"]</t>
+        </is>
+      </c>
       <c r="S37" t="inlineStr">
         <is>
           <t>level='本科' major=None</t>
         </is>
       </c>
-      <c r="T37" t="inlineStr"/>
       <c r="U37" t="inlineStr">
         <is>
           <t>["负责UE引擎中战斗系统的开发与迭代", "参与基础架构系统的设计与实现", "协同策划美术等团队调优战斗表现", "设计模块划分与数据流保障代码质量", "优化游戏运行性能包括内存渲染加载"]</t>
         </is>
       </c>
-      <c r="V37" t="inlineStr"/>
-      <c r="W37" t="inlineStr"/>
-      <c r="X37" t="inlineStr"/>
-      <c r="Y37" t="inlineStr"/>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>["负责UE引擎中战斗系统的开发与迭代", "参与基础架构系统的设计与实现", "协同策划美术等团队调优战斗表现", "设计模块划分与数据流保障代码质量", "优化游戏运行性能包括内存渲染加载"]</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4126,35 +4673,46 @@
 申请岗位</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr">
         <is>
           <t>["C++", "Lua", "UE", "任务"]</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr"/>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>["C++", "Lua", "UE", "任务"]</t>
+        </is>
+      </c>
       <c r="O38" t="inlineStr">
         <is>
           <t>["Lua", "UE"]</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr"/>
-      <c r="S38" t="inlineStr"/>
-      <c r="T38" t="inlineStr"/>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>["Lua", "UE"]</t>
+        </is>
+      </c>
       <c r="U38" t="inlineStr">
         <is>
           <t>["负责UE引擎中游戏任务系统开发与迭代", "参与基础架构系统设计与实现", "协同策划美术等团队调优任务系统", "设计模块划分与数据流保障代码质量", "针对游戏运行性能进行优化"]</t>
         </is>
       </c>
-      <c r="V38" t="inlineStr"/>
-      <c r="W38" t="inlineStr"/>
-      <c r="X38" t="inlineStr"/>
-      <c r="Y38" t="inlineStr"/>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>["负责UE引擎中游戏任务系统开发与迭代", "参与基础架构系统设计与实现", "协同策划美术等团队调优任务系统", "设计模块划分与数据流保障代码质量", "针对游戏运行性能进行优化"]</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4210,35 +4768,46 @@
 5、具备较强的结构化表达、指标分析和跨团队推进能力；能够将复杂技术问题转化为清晰的产品方案、决策依据和交付标准。</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr">
         <is>
           <t>["MLOps", "DevOps", "云原生", "AI应用", "机器学习"]</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr"/>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>["MLOps", "DevOps", "云原生", "AI应用", "机器学习"]</t>
+        </is>
+      </c>
       <c r="O39" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr"/>
-      <c r="S39" t="inlineStr"/>
-      <c r="T39" t="inlineStr"/>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="U39" t="inlineStr">
         <is>
           <t>["负责机器学习管理平台产品规划与版本设计", "深入业务场景识别效率质量稳定性问题", "负责平台能力设计（实验管理/训练编排/模型版本等）", "建立平台对象模型、状态流转和规则体系", "定义并跟踪关键产品指标，撰写PRD与验收标准"]</t>
         </is>
       </c>
-      <c r="V39" t="inlineStr"/>
-      <c r="W39" t="inlineStr"/>
-      <c r="X39" t="inlineStr"/>
-      <c r="Y39" t="inlineStr"/>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>["负责机器学习管理平台产品规划与版本设计", "深入业务场景识别效率质量稳定性问题", "负责平台能力设计（实验管理/训练编排/模型版本等）", "建立平台对象模型、状态流转和规则体系", "定义并跟踪关键产品指标，撰写PRD与验收标准"]</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=空）</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4293,35 +4862,46 @@
 5、有技术类项目管理工作经验的优先，不要求之前的工作经历一定是安全领域。</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr">
         <is>
           <t>["项目管理"]</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr"/>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>["项目管理"]</t>
+        </is>
+      </c>
       <c r="O40" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr"/>
-      <c r="S40" t="inlineStr"/>
-      <c r="T40" t="inlineStr"/>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="U40" t="inlineStr">
         <is>
           <t>["负责安全工程部门技术项目交付", "推动安全技术产品能力落地", "搭建项目管理流程与里程碑设定", "设计研发项目管理流程与工具"]</t>
         </is>
       </c>
-      <c r="V40" t="inlineStr"/>
-      <c r="W40" t="inlineStr"/>
-      <c r="X40" t="inlineStr"/>
-      <c r="Y40" t="inlineStr"/>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>["负责安全工程部门技术项目交付", "推动安全技术产品能力落地", "搭建项目管理流程与里程碑设定", "设计研发项目管理流程与工具"]</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=空）</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4377,35 +4957,46 @@
 5、具备Agent编写与应用能力，能够结合不同业务场景开展深入分析与运营提效。</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr">
         <is>
           <t>["SQL", "AGENT"]</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr"/>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>["SQL", "AGENT"]</t>
+        </is>
+      </c>
       <c r="O41" t="inlineStr">
         <is>
           <t>["SQL"]</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
-      <c r="T41" t="inlineStr"/>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>["SQL"]</t>
+        </is>
+      </c>
       <c r="U41" t="inlineStr">
         <is>
           <t>["搭建体验洞察到监控落地的全流程运营机制", "分析商家咨询数据识别经营与体验症结", "推动商家问题专项治理与持续改善", "前置评估运营策略与产品功能风险", "建立商家体验关键指标体系与监控闭环"]</t>
         </is>
       </c>
-      <c r="V41" t="inlineStr"/>
-      <c r="W41" t="inlineStr"/>
-      <c r="X41" t="inlineStr"/>
-      <c r="Y41" t="inlineStr"/>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>["搭建体验洞察到监控落地的全流程运营机制", "分析商家咨询数据识别经营与体验症结", "推动商家问题专项治理与持续改善", "前置评估运营策略与产品功能风险", "建立商家体验关键指标体系与监控闭环"]</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4460,35 +5051,46 @@
 4、有良好的资源协调与沟通能力，需要有效整合算法、产品、审核等多方资源，有推动复杂项目落地并拿到实际结果的经验。</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr">
         <is>
           <t>["SQL", "数据分析"]</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr"/>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>["SQL", "数据分析"]</t>
+        </is>
+      </c>
       <c r="O42" t="inlineStr">
         <is>
           <t>["电商治理策略", "风控", "策略运营", "规则制定", "商品审核", "内容审核"]</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr"/>
-      <c r="S42" t="inlineStr"/>
-      <c r="T42" t="inlineStr"/>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>["电商治理策略", "风控", "策略运营", "规则制定", "商品审核", "内容审核"]</t>
+        </is>
+      </c>
       <c r="U42" t="inlineStr">
         <is>
           <t>["负责耐消行业商品及内容风险治理", "搭建优化行业治理规则体系", "发掘风险问题并设计治理方案", "建立分层处置与闭环管控机制", "设计指标监控体系保障风险可控"]</t>
         </is>
       </c>
-      <c r="V42" t="inlineStr"/>
-      <c r="W42" t="inlineStr"/>
-      <c r="X42" t="inlineStr"/>
-      <c r="Y42" t="inlineStr"/>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>["负责耐消行业商品及内容风险治理", "搭建优化行业治理规则体系", "发掘风险问题并设计治理方案", "建立分层处置与闭环管控机制", "设计指标监控体系保障风险可控"]</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4550,39 +5152,56 @@
 4、有LLM-as-a-Judge、一致性校准、自动判分器、合成数据或评测集治理经验。</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr">
         <is>
           <t>["Python", "大语言模型", "AGENT", "Coding", "检索增强生成", "多轮对话", "评测Pipeline", "数据分析", "指标", "LLM-as-a-Judge"]</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr"/>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>["Python", "大语言模型", "AGENT", "Coding", "检索增强生成", "多轮对话", "评测Pipeline", "数据分析", "指标", "LLM-as-a-Judge"]</t>
+        </is>
+      </c>
       <c r="O43" t="inlineStr">
         <is>
           <t>["LLM-as-a-Judge", "OpenAI Evals", "LangSmith", "Langfuse", "RAGAS", "DeepEval", "SWE-bench", "HumanEval"]</t>
         </is>
       </c>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr"/>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>["LLM-as-a-Judge", "OpenAI Evals", "LangSmith", "Langfuse", "RAGAS", "DeepEval", "SWE-bench", "HumanEval"]</t>
+        </is>
+      </c>
       <c r="S43" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T43" t="inlineStr"/>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U43" t="inlineStr">
         <is>
           <t>["深入理解企业客户大模型应用场景，抽象评测任务", "建设端到端评测Pipeline覆盖复杂链路", "设计结果与过程指标定位模型失败环节", "分析评测结果与失败案例形成根因判断", "建设评测自动化与效率工具"]</t>
         </is>
       </c>
-      <c r="V43" t="inlineStr"/>
-      <c r="W43" t="inlineStr"/>
-      <c r="X43" t="inlineStr"/>
-      <c r="Y43" t="inlineStr"/>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>["深入理解企业客户大模型应用场景，抽象评测任务", "建设端到端评测Pipeline覆盖复杂链路", "设计结果与过程指标定位模型失败环节", "分析评测结果与失败案例形成根因判断", "建设评测自动化与效率工具"]</t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4637,35 +5256,46 @@
 5、善于沟通，有良好的团队协作能力，责任心。</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr">
         <is>
           <t>["关卡", "开放世界RPG", "MMORPG"]</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr"/>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>["关卡", "开放世界RPG", "MMORPG"]</t>
+        </is>
+      </c>
       <c r="O44" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr"/>
-      <c r="S44" t="inlineStr"/>
-      <c r="T44" t="inlineStr"/>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="U44" t="inlineStr">
         <is>
           <t>["负责游戏关卡相关设计，包括活动副本、场景交互解密探索、PVP竞技玩法", "与战斗、文案、系统、数值等环节策划合作优化关卡设计", "与程序合作研发、优化并维护关卡编辑器", "与美术合作跟进美术资产落地"]</t>
         </is>
       </c>
-      <c r="V44" t="inlineStr"/>
-      <c r="W44" t="inlineStr"/>
-      <c r="X44" t="inlineStr"/>
-      <c r="Y44" t="inlineStr"/>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>["负责游戏关卡相关设计，包括活动副本、场景交互解密探索、PVP竞技玩法", "与战斗、文案、系统、数值等环节策划合作优化关卡设计", "与程序合作研发、优化并维护关卡编辑器", "与美术合作跟进美术资产落地"]</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=空）</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4720,35 +5350,46 @@
 5、具备较强的目标感、跨部门沟通协作能力，能够高效联动产品、策略等相关方推进方案落地，并对结果持续跟进和复盘。</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr">
         <is>
           <t>["流程", "流程诊断", "数据分析", "问题归因", "AI工具", "产品思维"]</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr"/>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>["流程", "流程诊断", "数据分析", "问题归因", "AI工具", "产品思维"]</t>
+        </is>
+      </c>
       <c r="O45" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr"/>
-      <c r="S45" t="inlineStr"/>
-      <c r="T45" t="inlineStr"/>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="U45" t="inlineStr">
         <is>
           <t>["负责商家服务流程体系设计与优化", "推动AI能力在服务流程场景落地", "识别服务流程无效流转问题", "迭代服务流程产品工具与运营机制"]</t>
         </is>
       </c>
-      <c r="V45" t="inlineStr"/>
-      <c r="W45" t="inlineStr"/>
-      <c r="X45" t="inlineStr"/>
-      <c r="Y45" t="inlineStr"/>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>["负责商家服务流程体系设计与优化", "推动AI能力在服务流程场景落地", "识别服务流程无效流转问题", "迭代服务流程产品工具与运营机制"]</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=空）</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4801,39 +5442,56 @@
 4、具备数据分析经验，有用户增长、营销分析、商业分析经验者优先。</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr">
         <is>
           <t>["Hive", "MySQL", "数据分析", "Excel", "Tableau"]</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr"/>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>["Hive", "MySQL", "数据分析", "Excel", "Tableau"]</t>
+        </is>
+      </c>
       <c r="O46" t="inlineStr">
         <is>
           <t>["用户增长", "营销分析", "商业分析"]</t>
         </is>
       </c>
-      <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr"/>
-      <c r="R46" t="inlineStr"/>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>["用户增长", "营销分析", "商业分析"]</t>
+        </is>
+      </c>
       <c r="S46" t="inlineStr">
         <is>
           <t>level='本科' major='统计学'</t>
         </is>
       </c>
-      <c r="T46" t="inlineStr"/>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U46" t="inlineStr">
         <is>
           <t>["分析和迭代重点营销频道运营策略", "分析和迭代大促商城运营策略", "完善看数体系和自动化链路", "搭建标签体系和指标监控体系"]</t>
         </is>
       </c>
-      <c r="V46" t="inlineStr"/>
-      <c r="W46" t="inlineStr"/>
-      <c r="X46" t="inlineStr"/>
-      <c r="Y46" t="inlineStr"/>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>["分析和迭代重点营销频道运营策略", "分析和迭代大促商城运营策略", "完善看数体系和自动化链路", "搭建标签体系和指标监控体系"]</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4888,35 +5546,46 @@
 5、具备良好的沟通能力、优秀的项目管理和利益相关团队管理的能力，有过驱动复杂、跨团队合作经验的优先考虑。</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr">
         <is>
           <t>["数据分析"]</t>
         </is>
       </c>
-      <c r="N47" t="inlineStr"/>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>["数据分析"]</t>
+        </is>
+      </c>
       <c r="O47" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
-      <c r="R47" t="inlineStr"/>
-      <c r="S47" t="inlineStr"/>
-      <c r="T47" t="inlineStr"/>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="U47" t="inlineStr">
         <is>
           <t>["负责电商货架场景的玩法产品运营", "优化用户分层与补贴策略运营", "协同产品、数据分析、研发团队优化产品功能", "跨部门协作扩大业务收益", "监控市场变化制定增长策略"]</t>
         </is>
       </c>
-      <c r="V47" t="inlineStr"/>
-      <c r="W47" t="inlineStr"/>
-      <c r="X47" t="inlineStr"/>
-      <c r="Y47" t="inlineStr"/>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>["负责电商货架场景的玩法产品运营", "优化用户分层与补贴策略运营", "协同产品、数据分析、研发团队优化产品功能", "跨部门协作扩大业务收益", "监控市场变化制定增长策略"]</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=空）</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4976,35 +5645,46 @@
 6、有前端开发基础，能与研发高效对接，且对AI/AIGC在内容创作或互动场景中的应用有实践或浓厚兴趣。</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr">
         <is>
           <t>["交互", "视觉", "AIGC", "AGENT"]</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr"/>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>["交互", "视觉", "AIGC", "AGENT"]</t>
+        </is>
+      </c>
       <c r="O48" t="inlineStr">
         <is>
           <t>["动效"]</t>
         </is>
       </c>
-      <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="inlineStr"/>
-      <c r="S48" t="inlineStr"/>
-      <c r="T48" t="inlineStr"/>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>["动效"]</t>
+        </is>
+      </c>
       <c r="U48" t="inlineStr">
         <is>
           <t>["负责TikTok直播社交互动体验设计", "设计激发用户参与感的互动玩法", "梳理用户流程并输出交互方案与视觉落地"]</t>
         </is>
       </c>
-      <c r="V48" t="inlineStr"/>
-      <c r="W48" t="inlineStr"/>
-      <c r="X48" t="inlineStr"/>
-      <c r="Y48" t="inlineStr"/>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>["负责TikTok直播社交互动体验设计", "设计激发用户参与感的互动玩法", "梳理用户流程并输出交互方案与视觉落地"]</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5062,39 +5742,56 @@
 3、熟悉CDN、直播、RTC或其他边缘流量生产架构。</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr">
         <is>
           <t>["Go", "Python", "Linux", "存储", "容器", "Kubernetes", "虚拟化", "分布式技术", "云原生", "CDN", "RTC"]</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr"/>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>["Go", "Python", "Linux", "存储", "容器", "Kubernetes", "虚拟化", "分布式技术", "云原生", "CDN", "RTC"]</t>
+        </is>
+      </c>
       <c r="O49" t="inlineStr">
         <is>
           <t>["Containerd", "Cilium", "eBPF", "CDN", "RTC"]</t>
         </is>
       </c>
-      <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="inlineStr"/>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>["Containerd", "Cilium", "eBPF", "CDN", "RTC"]</t>
+        </is>
+      </c>
       <c r="S49" t="inlineStr">
         <is>
           <t>level='本科' major='计算机'</t>
         </is>
       </c>
-      <c r="T49" t="inlineStr"/>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U49" t="inlineStr">
         <is>
           <t>["设计构建全球边缘接入点基础设施组件", "建设高性能高可用可扩展基础设施系统", "保障多地域多租户场景稳定运行与资源交付", "与SRE平台产品团队协作提供平台能力"]</t>
         </is>
       </c>
-      <c r="V49" t="inlineStr"/>
-      <c r="W49" t="inlineStr"/>
-      <c r="X49" t="inlineStr"/>
-      <c r="Y49" t="inlineStr"/>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>["设计构建全球边缘接入点基础设施组件", "建设高性能高可用可扩展基础设施系统", "保障多地域多租户场景稳定运行与资源交付", "与SRE平台产品团队协作提供平台能力"]</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=硕士 bonus=LLM）；education 修正：原文「学士/硕士」门槛取本科</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5148,35 +5845,46 @@
 5、具备高熟练度的多语言能力，尤其是日语和英语。</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr">
         <is>
           <t>["世界观设定", "角色设定", "日语"]</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr"/>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>["世界观设定", "角色设定", "日语"]</t>
+        </is>
+      </c>
       <c r="O50" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
-      <c r="R50" t="inlineStr"/>
-      <c r="S50" t="inlineStr"/>
-      <c r="T50" t="inlineStr"/>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="U50" t="inlineStr">
         <is>
           <t>["撰写游戏世界观设定", "撰写主线与角色剧情大纲", "独立完成角色设定", "跟进资源制作流程"]</t>
         </is>
       </c>
-      <c r="V50" t="inlineStr"/>
-      <c r="W50" t="inlineStr"/>
-      <c r="X50" t="inlineStr"/>
-      <c r="Y50" t="inlineStr"/>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>["撰写游戏世界观设定", "撰写主线与角色剧情大纲", "独立完成角色设定", "跟进资源制作流程"]</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=空 bonus=空）</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5231,39 +5939,56 @@
 3、有直播、短视频、社区等内容生态相关工作经验者优先。</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr">
         <is>
           <t>["数据分析", "策略评估", "A/B测试", "大语言模型", "提示工程", "检索增强生成", "模型评估"]</t>
         </is>
       </c>
-      <c r="N51" t="inlineStr"/>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>["数据分析", "策略评估", "A/B测试", "大语言模型", "提示工程", "检索增强生成", "模型评估"]</t>
+        </is>
+      </c>
       <c r="O51" t="inlineStr">
         <is>
           <t>["AI", "Workflow搭建", "Agentic AI", "AI Workflow"]</t>
         </is>
       </c>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="inlineStr"/>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>["AI", "Workflow搭建", "Agentic AI", "AI Workflow"]</t>
+        </is>
+      </c>
       <c r="S51" t="inlineStr">
         <is>
           <t>level='本科' major=None</t>
         </is>
       </c>
-      <c r="T51" t="inlineStr"/>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
       <c r="U51" t="inlineStr">
         <is>
           <t>["负责直播经营情况分析与政策设计", "建立主播成长方法论框架", "搭建策略评估体系与数据建设", "协同运营算法工程团队推动策略落地", "通过A/B测试验证策略效果", "开展专题研究与用户调研"]</t>
         </is>
       </c>
-      <c r="V51" t="inlineStr"/>
-      <c r="W51" t="inlineStr"/>
-      <c r="X51" t="inlineStr"/>
-      <c r="Y51" t="inlineStr"/>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>["负责直播经营情况分析与政策设计", "建立主播成长方法论框架", "搭建策略评估体系与数据建设", "协同运营算法工程团队推动策略落地", "通过A/B测试验证策略效果", "开展专题研究与用户调研"]</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>auto（默认口径；education=本科 bonus=LLM）</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>